<commit_message>
student login, qr scan, verification page
</commit_message>
<xml_diff>
--- a/public/sample_students.xlsx
+++ b/public/sample_students.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Authblock\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4B62A0-DE11-4D0E-A35A-5CEFC64E7B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A949A69F-5F7B-4CCF-9806-FEC1FFD17305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="120">
   <si>
     <t>serial_no</t>
   </si>
@@ -250,9 +250,6 @@
     <t>sub_11_cpgp</t>
   </si>
   <si>
-    <t>Bachelor of Engineering Sem-IV</t>
-  </si>
-  <si>
     <t>Computer Engineering</t>
   </si>
   <si>
@@ -376,13 +373,13 @@
     <t>9.20</t>
   </si>
   <si>
-    <t>2023016400968411</t>
-  </si>
-  <si>
-    <t>SN-002</t>
-  </si>
-  <si>
-    <t>Raj Shamani</t>
+    <t>Bachelor of Engineering Sem-V</t>
+  </si>
+  <si>
+    <t>SN-0016</t>
+  </si>
+  <si>
+    <t>Alan Dsouza</t>
   </si>
 </sst>
 </file>
@@ -762,6 +759,7 @@
   <dimension ref="A1:BX2"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="3" width="23.625" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
   </cols>
   <sheetData>
@@ -997,236 +995,237 @@
     </row>
     <row r="2" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" t="s">
         <v>119</v>
       </c>
-      <c r="B2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" t="s">
-        <v>118</v>
+      <c r="C2">
+        <v>2023015400968420</v>
       </c>
       <c r="D2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E2" t="s">
         <v>76</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>77</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I2" t="s">
         <v>78</v>
       </c>
-      <c r="G2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H2" t="s">
-        <v>116</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>79</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>80</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>81</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>82</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
+        <v>97</v>
+      </c>
+      <c r="O2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P2" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q2" t="s">
         <v>83</v>
       </c>
-      <c r="N2" t="s">
+      <c r="R2" t="s">
+        <v>84</v>
+      </c>
+      <c r="S2" t="s">
+        <v>82</v>
+      </c>
+      <c r="T2" t="s">
+        <v>87</v>
+      </c>
+      <c r="U2" t="s">
+        <v>88</v>
+      </c>
+      <c r="V2" t="s">
+        <v>89</v>
+      </c>
+      <c r="W2" t="s">
+        <v>85</v>
+      </c>
+      <c r="X2" t="s">
+        <v>86</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>82</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>92</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>82</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>104</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>113</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>96</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>97</v>
+      </c>
+      <c r="AS2" t="s">
         <v>98</v>
       </c>
-      <c r="O2" t="s">
+      <c r="AT2" t="s">
+        <v>98</v>
+      </c>
+      <c r="AU2" t="s">
         <v>99</v>
       </c>
-      <c r="P2" t="s">
-        <v>115</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>84</v>
-      </c>
-      <c r="R2" t="s">
-        <v>85</v>
-      </c>
-      <c r="S2" t="s">
-        <v>83</v>
-      </c>
-      <c r="T2" t="s">
+      <c r="AV2" t="s">
+        <v>100</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>96</v>
+      </c>
+      <c r="AX2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AY2" t="s">
         <v>88</v>
       </c>
-      <c r="U2" t="s">
-        <v>89</v>
-      </c>
-      <c r="V2" t="s">
-        <v>90</v>
-      </c>
-      <c r="W2" t="s">
-        <v>86</v>
-      </c>
-      <c r="X2" t="s">
+      <c r="AZ2" t="s">
+        <v>88</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>101</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>102</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>96</v>
+      </c>
+      <c r="BD2" t="s">
         <v>87</v>
       </c>
-      <c r="Y2" t="s">
-        <v>83</v>
-      </c>
-      <c r="Z2" t="s">
+      <c r="BE2" t="s">
         <v>88</v>
       </c>
-      <c r="AA2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>83</v>
-      </c>
-      <c r="AF2" t="s">
+      <c r="BF2" t="s">
         <v>88</v>
       </c>
-      <c r="AG2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>93</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>83</v>
-      </c>
-      <c r="AL2" t="s">
+      <c r="BG2" t="s">
+        <v>105</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>106</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>96</v>
+      </c>
+      <c r="BJ2" t="s">
+        <v>97</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>98</v>
+      </c>
+      <c r="BL2" t="s">
+        <v>98</v>
+      </c>
+      <c r="BM2" t="s">
+        <v>107</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>108</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>109</v>
+      </c>
+      <c r="BP2" t="s">
+        <v>103</v>
+      </c>
+      <c r="BQ2" t="s">
         <v>104</v>
       </c>
-      <c r="AM2" t="s">
-        <v>105</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>114</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>95</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>96</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>97</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>98</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>99</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>99</v>
-      </c>
-      <c r="AU2" t="s">
-        <v>100</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>101</v>
-      </c>
-      <c r="AW2" t="s">
-        <v>97</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>89</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>102</v>
-      </c>
-      <c r="BB2" t="s">
+      <c r="BR2" t="s">
+        <v>112</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>111</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>109</v>
+      </c>
+      <c r="BV2" t="s">
         <v>103</v>
       </c>
-      <c r="BC2" t="s">
-        <v>97</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>89</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>89</v>
-      </c>
-      <c r="BG2" t="s">
-        <v>106</v>
-      </c>
-      <c r="BH2" t="s">
-        <v>107</v>
-      </c>
-      <c r="BI2" t="s">
-        <v>97</v>
-      </c>
-      <c r="BJ2" t="s">
-        <v>98</v>
-      </c>
-      <c r="BK2" t="s">
-        <v>99</v>
-      </c>
-      <c r="BL2" t="s">
-        <v>99</v>
-      </c>
-      <c r="BM2" t="s">
-        <v>108</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>109</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>110</v>
-      </c>
-      <c r="BP2" t="s">
+      <c r="BW2" t="s">
         <v>104</v>
       </c>
-      <c r="BQ2" t="s">
-        <v>105</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>113</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>111</v>
-      </c>
-      <c r="BT2" t="s">
+      <c r="BX2" t="s">
         <v>112</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>110</v>
-      </c>
-      <c r="BV2" t="s">
-        <v>104</v>
-      </c>
-      <c r="BW2" t="s">
-        <v>105</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>113</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A1:BX1" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Marksheet Data Extraction & Verification
</commit_message>
<xml_diff>
--- a/public/sample_students.xlsx
+++ b/public/sample_students.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Authblock\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EAA8BD4-75FB-41E6-811E-313A5515250B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69C7938-CB48-4340-BEE1-4808F87A469E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Marksheets" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="118">
   <si>
     <t>serial_no</t>
   </si>
@@ -367,19 +367,13 @@
     <t>28</t>
   </si>
   <si>
-    <t>9.10</t>
-  </si>
-  <si>
-    <t>9.20</t>
-  </si>
-  <si>
     <t>Bachelor of Engineering Sem-V</t>
   </si>
   <si>
     <t>SN-0016</t>
   </si>
   <si>
-    <t>Jaden Britto</t>
+    <t>Jake Suli</t>
   </si>
 </sst>
 </file>
@@ -757,13 +751,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BX2"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="23.59765625" customWidth="1"/>
+    <col min="3" max="3" width="23.625" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:76" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -993,18 +987,18 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:76" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:76" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C2">
-        <v>2023015400968430</v>
+        <v>2023015400968440</v>
       </c>
       <c r="D2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E2" t="s">
         <v>76</v>
@@ -1012,11 +1006,11 @@
       <c r="F2" t="s">
         <v>77</v>
       </c>
-      <c r="G2" t="s">
-        <v>116</v>
-      </c>
-      <c r="H2" t="s">
-        <v>115</v>
+      <c r="G2">
+        <v>8.75</v>
+      </c>
+      <c r="H2">
+        <v>8.8800000000000008</v>
       </c>
       <c r="I2" t="s">
         <v>78</v>

</xml_diff>

<commit_message>
S3 & Email Input Config
</commit_message>
<xml_diff>
--- a/public/sample_students.xlsx
+++ b/public/sample_students.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Authblock\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69C7938-CB48-4340-BEE1-4808F87A469E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D9664D-B956-4847-8265-732DB9AA3A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="123">
   <si>
     <t>serial_no</t>
   </si>
@@ -28,6 +28,9 @@
     <t>student_name</t>
   </si>
   <si>
+    <t>student_email</t>
+  </si>
+  <si>
     <t>prn_no</t>
   </si>
   <si>
@@ -250,12 +253,21 @@
     <t>sub_11_cpgp</t>
   </si>
   <si>
+    <t>Bachelor of Engineering Sem-IV</t>
+  </si>
+  <si>
     <t>Computer Engineering</t>
   </si>
   <si>
     <t>June-2025</t>
   </si>
   <si>
+    <t>8.90</t>
+  </si>
+  <si>
+    <t>8.45</t>
+  </si>
+  <si>
     <t>SUCCESSFUL</t>
   </si>
   <si>
@@ -271,18 +283,42 @@
     <t>4</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
     <t>CSC402</t>
   </si>
   <si>
     <t>ANALYSIS OF ALGORITHMS</t>
   </si>
   <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
     <t>CSC403</t>
   </si>
   <si>
     <t>DATABASE MANAGEMENT</t>
   </si>
   <si>
+    <t>CSC404</t>
+  </si>
+  <si>
+    <t>OPERATING SYSTEMS</t>
+  </si>
+  <si>
     <t>B</t>
   </si>
   <si>
@@ -292,12 +328,6 @@
     <t>32</t>
   </si>
   <si>
-    <t>CSC404</t>
-  </si>
-  <si>
-    <t>OPERATING SYSTEMS</t>
-  </si>
-  <si>
     <t>CSC405</t>
   </si>
   <si>
@@ -313,12 +343,6 @@
     <t>1</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
     <t>CSL402</t>
   </si>
   <si>
@@ -331,12 +355,6 @@
     <t>OS LAB</t>
   </si>
   <si>
-    <t>O</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>CSL404</t>
   </si>
   <si>
@@ -352,6 +370,9 @@
     <t>2</t>
   </si>
   <si>
+    <t>14</t>
+  </si>
+  <si>
     <t>CSM401</t>
   </si>
   <si>
@@ -361,29 +382,31 @@
     <t>20</t>
   </si>
   <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>Bachelor of Engineering Sem-V</t>
-  </si>
-  <si>
-    <t>SN-0016</t>
-  </si>
-  <si>
-    <t>Jake Suli</t>
+    <t>SN-0026</t>
+  </si>
+  <si>
+    <t>jasonemail28@gmail.com</t>
+  </si>
+  <si>
+    <t>Ario Learner</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -406,13 +429,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -750,14 +776,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BX2"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BY11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="23.625" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="2" max="2" width="18.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:77" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -986,242 +1013,259 @@
       <c r="BX1" t="s">
         <v>75</v>
       </c>
+      <c r="BY1" t="s">
+        <v>76</v>
+      </c>
     </row>
-    <row r="2" spans="1:76" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:77" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C2">
-        <v>2023015400968440</v>
-      </c>
-      <c r="D2" t="s">
-        <v>115</v>
+        <v>122</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2">
+        <v>2023016400968460</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G2">
-        <v>8.75</v>
-      </c>
-      <c r="H2">
-        <v>8.8800000000000008</v>
+        <v>78</v>
+      </c>
+      <c r="G2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" t="s">
+        <v>80</v>
       </c>
       <c r="I2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="J2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="K2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="L2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="M2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="N2" t="s">
+        <v>86</v>
+      </c>
+      <c r="O2" t="s">
+        <v>87</v>
+      </c>
+      <c r="P2" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>89</v>
+      </c>
+      <c r="R2" t="s">
+        <v>90</v>
+      </c>
+      <c r="S2" t="s">
+        <v>91</v>
+      </c>
+      <c r="T2" t="s">
+        <v>86</v>
+      </c>
+      <c r="U2" t="s">
+        <v>92</v>
+      </c>
+      <c r="V2" t="s">
+        <v>93</v>
+      </c>
+      <c r="W2" t="s">
+        <v>94</v>
+      </c>
+      <c r="X2" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>96</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AD2" t="s">
         <v>97</v>
       </c>
-      <c r="O2" t="s">
+      <c r="AE2" t="s">
         <v>98</v>
       </c>
-      <c r="P2" t="s">
-        <v>114</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>83</v>
-      </c>
-      <c r="R2" t="s">
-        <v>84</v>
-      </c>
-      <c r="S2" t="s">
-        <v>82</v>
-      </c>
-      <c r="T2" t="s">
-        <v>87</v>
-      </c>
-      <c r="U2" t="s">
-        <v>88</v>
-      </c>
-      <c r="V2" t="s">
-        <v>89</v>
-      </c>
-      <c r="W2" t="s">
-        <v>85</v>
-      </c>
-      <c r="X2" t="s">
+      <c r="AF2" t="s">
         <v>86</v>
       </c>
-      <c r="Y2" t="s">
-        <v>82</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>91</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AF2" t="s">
-        <v>87</v>
-      </c>
       <c r="AG2" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="AH2" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="AI2" t="s">
+        <v>101</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>103</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AM2" t="s">
         <v>92</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AN2" t="s">
         <v>93</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>82</v>
-      </c>
-      <c r="AL2" t="s">
-        <v>103</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>104</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>113</v>
       </c>
       <c r="AO2" t="s">
         <v>94</v>
       </c>
       <c r="AP2" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="AQ2" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="AR2" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="AS2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="AT2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="AU2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="AV2" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="AW2" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="AX2" t="s">
+        <v>106</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>92</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>93</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>93</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>109</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>110</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>106</v>
+      </c>
+      <c r="BE2" t="s">
         <v>87</v>
-      </c>
-      <c r="AY2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>88</v>
-      </c>
-      <c r="BA2" t="s">
-        <v>101</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>102</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>96</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>87</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>88</v>
       </c>
       <c r="BF2" t="s">
         <v>88</v>
       </c>
       <c r="BG2" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="BH2" t="s">
+        <v>111</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>112</v>
+      </c>
+      <c r="BJ2" t="s">
         <v>106</v>
       </c>
-      <c r="BI2" t="s">
-        <v>96</v>
-      </c>
-      <c r="BJ2" t="s">
-        <v>97</v>
-      </c>
       <c r="BK2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="BL2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="BM2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="BN2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="BO2" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="BP2" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="BQ2" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="BR2" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="BS2" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="BT2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="BU2" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="BV2" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="BW2" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="BX2" t="s">
-        <v>112</v>
+        <v>88</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>119</v>
       </c>
     </row>
+    <row r="3" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:77" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{D343730C-B31C-4718-B06D-F4B67DD39F16}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:BX1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:BY1 E2:BY2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Edge Detection of Doc
</commit_message>
<xml_diff>
--- a/public/sample_students.xlsx
+++ b/public/sample_students.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Authblock\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{131CF2E8-F46F-4E7A-ABE2-8208B6C32720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1D39DC-CDE3-419D-BFBA-4CCD7EC1ED20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -373,13 +373,13 @@
     <t>jasonemail28@gmail.com</t>
   </si>
   <si>
-    <t>SN-0045</t>
-  </si>
-  <si>
-    <t>Sam Altman</t>
-  </si>
-  <si>
-    <t>Bachelor of Engineering Sem IV</t>
+    <t>Ario Learner</t>
+  </si>
+  <si>
+    <t>Bachelor of Engineering Sem Testnew</t>
+  </si>
+  <si>
+    <t>SN-0047</t>
   </si>
 </sst>
 </file>
@@ -1011,19 +1011,19 @@
     </row>
     <row r="2" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" t="s">
         <v>117</v>
-      </c>
-      <c r="B2" t="s">
-        <v>118</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>116</v>
       </c>
       <c r="D2">
-        <v>2023015400968440</v>
+        <v>2023016400968460</v>
       </c>
       <c r="E2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F2" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
amplify domain for image
</commit_message>
<xml_diff>
--- a/public/sample_students.xlsx
+++ b/public/sample_students.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Authblock\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90706925-947B-4109-B639-17EB66DF2C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B65468-FBB3-443F-8EE2-8E0735BD5888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Marksheets" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="120">
   <si>
     <t>serial_no</t>
   </si>
@@ -373,22 +373,13 @@
     <t>jasonemail28@gmail.com</t>
   </si>
   <si>
-    <t>Ario Learner</t>
-  </si>
-  <si>
     <t>Sam Altman</t>
   </si>
   <si>
-    <t>SN-0049</t>
-  </si>
-  <si>
-    <t>SN-0050</t>
-  </si>
-  <si>
-    <t>morganforgemorganforge@gmail.com</t>
-  </si>
-  <si>
     <t>Bachelor of Engineering Sem V</t>
+  </si>
+  <si>
+    <t>SN-0105</t>
   </si>
 </sst>
 </file>
@@ -1023,7 +1014,7 @@
         <v>119</v>
       </c>
       <c r="B2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>116</v>
@@ -1032,7 +1023,7 @@
         <v>2023016400968440</v>
       </c>
       <c r="E2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F2" t="s">
         <v>77</v>
@@ -1252,242 +1243,12 @@
       </c>
     </row>
     <row r="3" spans="1:77" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D3">
-        <v>2023016400968460</v>
-      </c>
-      <c r="E3" t="s">
-        <v>122</v>
-      </c>
-      <c r="F3" t="s">
-        <v>77</v>
-      </c>
-      <c r="G3" s="2">
-        <v>46174</v>
-      </c>
-      <c r="H3">
-        <v>7.45</v>
-      </c>
-      <c r="I3">
-        <v>8.25</v>
-      </c>
-      <c r="J3" t="s">
-        <v>78</v>
-      </c>
-      <c r="K3" t="s">
-        <v>79</v>
-      </c>
-      <c r="L3" t="s">
-        <v>80</v>
-      </c>
-      <c r="M3" t="s">
-        <v>81</v>
-      </c>
-      <c r="N3" t="s">
-        <v>82</v>
-      </c>
-      <c r="O3" t="s">
-        <v>83</v>
-      </c>
-      <c r="P3" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>85</v>
-      </c>
-      <c r="R3" t="s">
-        <v>86</v>
-      </c>
-      <c r="S3" t="s">
-        <v>87</v>
-      </c>
-      <c r="T3" t="s">
-        <v>82</v>
-      </c>
-      <c r="U3" t="s">
-        <v>88</v>
-      </c>
-      <c r="V3" t="s">
-        <v>89</v>
-      </c>
-      <c r="W3" t="s">
-        <v>90</v>
-      </c>
-      <c r="X3" t="s">
-        <v>91</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>92</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>83</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>85</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>82</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>96</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>97</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>99</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>82</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>89</v>
-      </c>
-      <c r="AO3" t="s">
-        <v>90</v>
-      </c>
-      <c r="AP3" t="s">
-        <v>100</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>101</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>102</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>89</v>
-      </c>
-      <c r="AU3" t="s">
-        <v>89</v>
-      </c>
-      <c r="AV3" t="s">
-        <v>103</v>
-      </c>
-      <c r="AW3" t="s">
-        <v>104</v>
-      </c>
-      <c r="AX3" t="s">
-        <v>102</v>
-      </c>
-      <c r="AY3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AZ3" t="s">
-        <v>89</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>89</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>105</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>106</v>
-      </c>
-      <c r="BD3" t="s">
-        <v>102</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>83</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>84</v>
-      </c>
-      <c r="BG3" t="s">
-        <v>84</v>
-      </c>
-      <c r="BH3" t="s">
-        <v>107</v>
-      </c>
-      <c r="BI3" t="s">
-        <v>108</v>
-      </c>
-      <c r="BJ3" t="s">
-        <v>102</v>
-      </c>
-      <c r="BK3" t="s">
-        <v>95</v>
-      </c>
-      <c r="BL3" t="s">
-        <v>96</v>
-      </c>
-      <c r="BM3" t="s">
-        <v>96</v>
-      </c>
-      <c r="BN3" t="s">
-        <v>109</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>110</v>
-      </c>
-      <c r="BP3" t="s">
-        <v>111</v>
-      </c>
-      <c r="BQ3" t="s">
-        <v>88</v>
-      </c>
-      <c r="BR3" t="s">
-        <v>89</v>
-      </c>
-      <c r="BS3" t="s">
-        <v>112</v>
-      </c>
-      <c r="BT3" t="s">
-        <v>113</v>
-      </c>
-      <c r="BU3" t="s">
-        <v>114</v>
-      </c>
-      <c r="BV3" t="s">
-        <v>111</v>
-      </c>
-      <c r="BW3" t="s">
-        <v>83</v>
-      </c>
-      <c r="BX3" t="s">
-        <v>84</v>
-      </c>
-      <c r="BY3" t="s">
-        <v>115</v>
-      </c>
+      <c r="C3" s="1"/>
+      <c r="G3" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{E0D25F5D-444E-4478-97FA-13C818FFD71B}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{D4F6B9F7-A43B-41FB-BA4F-543CC11BBB32}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>